<commit_message>
creates table with the right h2 datatypes
</commit_message>
<xml_diff>
--- a/src/main/resources/data.xlsx
+++ b/src/main/resources/data.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="cica" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="original" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,25 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+  <si>
+    <t xml:space="preserve">birth date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alma</t>
+  </si>
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -37,36 +56,53 @@
     <t xml:space="preserve">USA</t>
   </si>
   <si>
+    <t xml:space="preserve">2020.01.01</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bob</t>
   </si>
   <si>
     <t xml:space="preserve">Canada</t>
   </si>
   <si>
+    <t xml:space="preserve">2020.01.02</t>
+  </si>
+  <si>
     <t xml:space="preserve">Charlie</t>
   </si>
   <si>
     <t xml:space="preserve">UK</t>
   </si>
   <si>
+    <t xml:space="preserve">2020.01.03</t>
+  </si>
+  <si>
     <t xml:space="preserve">Diana</t>
   </si>
   <si>
     <t xml:space="preserve">Germany</t>
   </si>
   <si>
+    <t xml:space="preserve">2020.01.04</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ethan</t>
   </si>
   <si>
     <t xml:space="preserve">Australia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020.01.05</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -136,12 +172,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -268,74 +312,54 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
+      <c r="A2" s="2" t="n">
+        <v>43834</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>123</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>42.42</v>
+      </c>
+      <c r="E2" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="A3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="A6" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -346,4 +370,107 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Normál"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normál"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normál"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>